<commit_message>
Reformatacao da matriz de requsiitos
</commit_message>
<xml_diff>
--- a/DocumentacaoEngenharia/2SIR-ListaRequisitosSiEstacionamento.xlsx
+++ b/DocumentacaoEngenharia/2SIR-ListaRequisitosSiEstacionamento.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\renat\Downloads\MaterialAulasPDF\2SI-EngSw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A6B85B46-7922-4AEF-B201-CD29BCBBE494}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EBF029B-3613-4623-B162-1BC89C94D663}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{DAAFDAA2-2CA9-4C52-945F-588F58466B28}"/>
   </bookViews>
@@ -30,9 +30,6 @@
     <t>LISTA DE REQUISITOS - PROJETO DO SISTEMA DE ESTACIONAMENTO</t>
   </si>
   <si>
-    <t>Nome</t>
-  </si>
-  <si>
     <t>Descrição das regras de domínio</t>
   </si>
   <si>
@@ -41,12 +38,15 @@
   <si>
     <t>*Legenda: Rf = Requisito funcional; Rnf = Requisito não funcional</t>
   </si>
+  <si>
+    <t>Nome do requisito</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -61,8 +61,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -72,6 +80,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="3"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -103,10 +117,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -430,24 +446,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="4"/>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="s">
+      <c r="C4" s="2" t="s">
         <v>1</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Alteracao matriz de requisitos original recuperada
Alteracao da matriz de requisitos com base na copia original, recuperada.
</commit_message>
<xml_diff>
--- a/DocumentacaoEngenharia/2SIR-ListaRequisitosSiEstacionamento.xlsx
+++ b/DocumentacaoEngenharia/2SIR-ListaRequisitosSiEstacionamento.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\renat\Downloads\MaterialAulasPDF\2SI-EngSw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EBF029B-3613-4623-B162-1BC89C94D663}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BED5503-DBEB-4090-B4E5-80C9C0A7CDE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{DAAFDAA2-2CA9-4C52-945F-588F58466B28}"/>
   </bookViews>
@@ -36,17 +36,40 @@
     <t>Id*</t>
   </si>
   <si>
-    <t>*Legenda: Rf = Requisito funcional; Rnf = Requisito não funcional</t>
+    <t>Nome do requisito</t>
   </si>
   <si>
-    <t>Nome do requisito</t>
+    <r>
+      <t>*</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Legenda</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: Rf = Requisito funcional; Rnf = Requisito não funcional</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -55,6 +78,14 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="0"/>
       <name val="Calibri"/>
@@ -85,7 +116,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="3" tint="0.59999389629810485"/>
+        <fgColor theme="5" tint="-0.499984740745262"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -121,8 +152,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -452,7 +483,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B2" s="4"/>
     </row>
@@ -461,7 +492,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>1</v>

</xml_diff>